<commit_message>
feat(imports): add mapped bill/bill-payment imports and harden cash purchase posting
- add bill and bill-payment import pages with upload, field mapping, preview, and execute flows
- extend PurchaseController and BillPaymentsController for import session handling, validation previews, and execution
- add BillPaymentImport and refactor BillInvoiceImport to support mapped headers, grouped records, tax parsing, and resilient date parsing
- move imported purchase/bill accounting entries to pending transactions with approval/checker record creation
- enhance CashPurchaseImport with tax support and related purchase item tax records
- fix cash purchase create/edit line array alignment and add backend guard for misaligned line item payloads
- update bill/bill-payment UI entry points, add bill payment sample template, update bill sample, and show total due on bill payment view
</commit_message>
<xml_diff>
--- a/public/uploads/media/default/sample_bills.xlsx
+++ b/public/uploads/media/default/sample_bills.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohamedjagne\Desktop\Mohamed\Projects\sahardid1\public\uploads\media\default\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moham\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F803BD6-2B93-4B05-87E6-58977B0675DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA1DCB9-7206-44AC-8F0E-4D68DC926EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sample_bills" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>title</t>
   </si>
@@ -82,6 +93,18 @@
   </si>
   <si>
     <t>Bill invoice</t>
+  </si>
+  <si>
+    <t>bill_number</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>is_inventory</t>
+  </si>
+  <si>
+    <t>expense_account</t>
   </si>
 </sst>
 </file>
@@ -400,99 +423,119 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" customWidth="1"/>
+    <col min="11" max="11" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="4.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" t="s">
+      <c r="Q1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
         <v>17</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>45374</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>45376</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>11</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>0</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>5</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="M2" t="s">
         <v>12</v>
       </c>
-      <c r="K2">
+      <c r="O2">
         <v>12</v>
       </c>
-      <c r="L2">
+      <c r="P2">
         <v>18</v>
       </c>
-      <c r="M2" t="s">
+      <c r="Q2" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>